<commit_message>
Refresh stale market data before reporting
</commit_message>
<xml_diff>
--- a/reports/latest_one_month_follow_up.xlsx
+++ b/reports/latest_one_month_follow_up.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="TAKIP_OZETI" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="POZISYONLAR" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="GUNLUK_TAKIP" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="NOTLAR" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TAKIP_OZETI" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="POZISYONLAR" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GUNLUK_TAKIP" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NOTLAR" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TAKIP_OZETI'!$A$1:$B$16</definedName>
@@ -27,16 +27,13 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -56,7 +53,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -64,23 +61,14 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -464,186 +452,186 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="29" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Alan</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Değer</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Rapor Tarihi</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Strateji</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Top3 Ranking Only</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Rejim Durumu</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>ABOVE_MA200_RISK_ON</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>BIST100 Kapanış</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n">
-        <v>13704</v>
+      <c r="B5" s="3" t="n">
+        <v>14729.7001953125</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Portföy Başlangıç Değeri</t>
         </is>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="3" t="n">
         <v>100000</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Seçilen 3 Hisse</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>EREGL.IS, SISE.IS, BIMAS.IS</t>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>AKBNK.IS, YKBNK.IS, BIMAS.IS</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Eşit Ağırlık</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>33.33% / 33.33% / 33.33%</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Başlangıç Tarihi</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Güncel Fiyat Tarihi</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>BIST100 Başlangıç Tarihi</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>BIST100 Güncel Tarihi</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Portföy Toplam Getiri</t>
         </is>
       </c>
-      <c r="B13" s="4" t="n">
+      <c r="B13" s="3" t="n">
         <v>-1.110223024625157e-16</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>BIST100 Getiri</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="3" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>BIST100'e Göre Fark</t>
         </is>
       </c>
-      <c r="B15" s="4" t="n">
+      <c r="B15" s="3" t="n">
         <v>-1.110223024625157e-16</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Durum</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>Zararda / BIST Altı</t>
         </is>
@@ -666,8 +654,8 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="19" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
@@ -675,128 +663,128 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Hisse</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Ağırlık %</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Başlangıç Fiyatı</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Güncel Fiyat</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Getiri %</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Başlangıç Tutarı</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Güncel Tutar</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Kar/Zarar TL</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>EREGL.IS</t>
-        </is>
-      </c>
-      <c r="B2" s="5" t="n">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>AKBNK.IS</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="C2" s="6" t="n">
-        <v>40</v>
-      </c>
-      <c r="D2" s="6" t="n">
-        <v>40</v>
-      </c>
-      <c r="E2" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" s="6" t="n">
+      <c r="C2" s="5" t="n">
+        <v>82</v>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>82</v>
+      </c>
+      <c r="E2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="5" t="n">
         <v>33333.33333333333</v>
       </c>
-      <c r="G2" s="6" t="n">
+      <c r="G2" s="5" t="n">
         <v>33333.33333333333</v>
       </c>
-      <c r="H2" s="6" t="n">
+      <c r="H2" s="5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>SISE.IS</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="n">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>YKBNK.IS</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="C3" s="6" t="n">
-        <v>45.5</v>
-      </c>
-      <c r="D3" s="6" t="n">
-        <v>45.5</v>
-      </c>
-      <c r="E3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" s="6" t="n">
+      <c r="C3" s="5" t="n">
+        <v>43.84000015258789</v>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>43.84000015258789</v>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="5" t="n">
         <v>33333.33333333333</v>
       </c>
-      <c r="G3" s="6" t="n">
+      <c r="G3" s="5" t="n">
         <v>33333.33333333333</v>
       </c>
-      <c r="H3" s="6" t="n">
+      <c r="H3" s="5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>BIMAS.IS</t>
         </is>
       </c>
-      <c r="B4" s="5" t="n">
+      <c r="B4" s="4" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="C4" s="6" t="n">
-        <v>371.25</v>
-      </c>
-      <c r="D4" s="6" t="n">
-        <v>371.25</v>
-      </c>
-      <c r="E4" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="6" t="n">
+      <c r="C4" s="5" t="n">
+        <v>379</v>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>379</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="5" t="n">
         <v>33333.33333333333</v>
       </c>
-      <c r="G4" s="6" t="n">
+      <c r="G4" s="5" t="n">
         <v>33333.33333333333</v>
       </c>
-      <c r="H4" s="6" t="n">
+      <c r="H4" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -819,68 +807,68 @@
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Tarih</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Portföy Değeri</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Günlük Getiri %</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Toplam Getiri %</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>BIST100 Değeri</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>BIST100 Getiri %</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Fark %</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="n">
-        <v>46174</v>
-      </c>
-      <c r="B2" s="6" t="n">
+      <c r="A2" s="6" t="n">
+        <v>46195</v>
+      </c>
+      <c r="B2" s="5" t="n">
         <v>100000</v>
       </c>
-      <c r="C2" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D2" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" s="6" t="n">
-        <v>13704</v>
-      </c>
-      <c r="F2" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" s="5" t="n">
+      <c r="C2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>14729.7001953125</v>
+      </c>
+      <c r="F2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -903,42 +891,42 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Notlar</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Bu dosya araştırma dosyası değildir.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Bir aylık takip dosyasıdır.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Alım/satım önerisi değildir.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Amaç stratejinin BIST100’e göre performansını takip etmektir.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Bir ay boyunca aynı 3 hisse takip edilir.</t>
         </is>

</xml_diff>

<commit_message>
Fix one month follow-up tracking state
</commit_message>
<xml_diff>
--- a/reports/latest_one_month_follow_up.xlsx
+++ b/reports/latest_one_month_follow_up.xlsx
@@ -13,10 +13,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NOTLAR" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TAKIP_OZETI'!$A$1:$B$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TAKIP_OZETI'!$A$1:$B$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'POZISYONLAR'!$A$1:$H$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'GUNLUK_TAKIP'!$A$1:$G$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'NOTLAR'!$A$1:$A$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'GUNLUK_TAKIP'!$A$1:$G$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'NOTLAR'!$A$1:$A$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -448,11 +448,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="29" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -482,163 +482,199 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Strateji</t>
+          <t>Takip Modu</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Top3 Ranking Only</t>
+          <t>Sabit portföy</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Rejim Durumu</t>
+          <t>Strateji</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>ABOVE_MA200_RISK_ON</t>
+          <t>Top3 Ranking Only</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>BIST100 Kapanış</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>14729.7001953125</v>
+          <t>Başlangıç Modeli</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>volume_heavy</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Portföy Başlangıç Değeri</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="n">
-        <v>100000</v>
+          <t>Başlangıç Rejim Durumu</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>ABOVE_MA200_RISK_ON</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Seçilen 3 Hisse</t>
+          <t>Güncel Rejim Durumu</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>AKBNK.IS, YKBNK.IS, BIMAS.IS</t>
+          <t>ABOVE_MA200_RISK_ON</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Eşit Ağırlık</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>33.33% / 33.33% / 33.33%</t>
-        </is>
+          <t>BIST100 Kapanış</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>14729.7001953125</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Başlangıç Tarihi</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
+          <t>Portföy Başlangıç Değeri</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>100000</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Güncel Fiyat Tarihi</t>
+          <t>Seçilen 3 Hisse</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>EREGL.IS, SISE.IS, BIMAS.IS</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>BIST100 Başlangıç Tarihi</t>
+          <t>Eşit Ağırlık</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>33.33% / 33.33% / 33.33%</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>BIST100 Güncel Tarihi</t>
+          <t>Başlangıç Tarihi</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Portföy Toplam Getiri</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="n">
-        <v>-1.110223024625157e-16</v>
+          <t>Güncel Fiyat Tarihi</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>BIST100 Getiri</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="n">
-        <v>0</v>
+          <t>BIST100 Başlangıç Tarihi</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>BIST100'e Göre Fark</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="n">
-        <v>-1.110223024625157e-16</v>
+          <t>BIST100 Güncel Tarihi</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
+          <t>Portföy Toplam Getiri</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0.01579913200164529</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>BIST100 Getiri</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0.07484677432227826</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>BIST100'e Göre Fark</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>-0.05904764232063298</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
           <t>Durum</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>Zararda / BIST Altı</t>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Karda / BIST Altı</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B16"/>
+  <autoFilter ref="A1:B19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -654,12 +690,12 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="19" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -707,57 +743,57 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>AKBNK.IS</t>
+          <t>EREGL.IS</t>
         </is>
       </c>
       <c r="B2" s="4" t="n">
         <v>0.3333333333333333</v>
       </c>
       <c r="C2" s="5" t="n">
-        <v>82</v>
+        <v>40</v>
       </c>
       <c r="D2" s="5" t="n">
-        <v>82</v>
+        <v>40.34000015258789</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>0</v>
+        <v>0.008500003814697177</v>
       </c>
       <c r="F2" s="5" t="n">
         <v>33333.33333333333</v>
       </c>
       <c r="G2" s="5" t="n">
-        <v>33333.33333333333</v>
+        <v>33616.66679382323</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0</v>
+        <v>283.3334604899064</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>YKBNK.IS</t>
+          <t>SISE.IS</t>
         </is>
       </c>
       <c r="B3" s="4" t="n">
         <v>0.3333333333333333</v>
       </c>
       <c r="C3" s="5" t="n">
-        <v>43.84000015258789</v>
+        <v>45.5</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>43.84000015258789</v>
+        <v>46.31999969482422</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>0</v>
+        <v>0.01802197131481797</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>33333.33333333333</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>33333.33333333333</v>
+        <v>33934.06571049393</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>0</v>
+        <v>600.7323771606025</v>
       </c>
     </row>
     <row r="4">
@@ -770,22 +806,22 @@
         <v>0.3333333333333333</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>379</v>
+        <v>371.25</v>
       </c>
       <c r="D4" s="5" t="n">
         <v>379</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>0</v>
+        <v>0.02087542087542094</v>
       </c>
       <c r="F4" s="5" t="n">
         <v>33333.33333333333</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>33333.33333333333</v>
+        <v>34029.18069584736</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0</v>
+        <v>695.8473625140323</v>
       </c>
     </row>
   </sheetData>
@@ -800,16 +836,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -851,7 +887,7 @@
     </row>
     <row r="2">
       <c r="A2" s="6" t="n">
-        <v>46195</v>
+        <v>46174</v>
       </c>
       <c r="B2" s="5" t="n">
         <v>100000</v>
@@ -863,7 +899,7 @@
         <v>0</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>14729.7001953125</v>
+        <v>13704</v>
       </c>
       <c r="F2" s="4" t="n">
         <v>0</v>
@@ -872,8 +908,353 @@
         <v>0</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="6" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>102223.0027697347</v>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>0.02223002769734705</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>0.02223002769734705</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>14200.2001953125</v>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>0.03620842055695417</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>-0.01397839285960711</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>101548.9054270188</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>-0.006594380173260195</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>0.01548905427018843</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>13965.7001953125</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>0.01909662837948778</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>-0.00360757410929935</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>100052.2803667449</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>-0.01473797333393734</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>0.0005228036674491676</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>13872.2998046875</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>0.01228107156213509</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>-0.01175826789468593</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>99150.39483732327</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>-0.009014142667371106</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>-0.008496051626767365</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>13694.2001953125</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>-0.0007151054208625052</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>-0.00778094620590486</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>99194.90173474306</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>0.000448882704832565</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>-0.008050982652569316</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>13860.599609375</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>0.01142729198591641</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>-0.01947827463848573</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>98960.65707117392</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>-0.002361458698709518</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>-0.01039342928826081</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>13741.900390625</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>0.002765644383026844</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>-0.01315907367128766</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>98567.79623824963</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>-0.003969868880738581</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>-0.01432203761750372</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>13744.599609375</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>0.002962610141199695</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>-0.01728464775870342</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>97972.1929521213</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>-0.006042574845527504</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>-0.02027807047878705</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>13743.5</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>0.00288237011091641</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>-0.02316044058970346</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>99533.39140527607</v>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>0.01593511797697267</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>-0.004666085947239274</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>13938.5</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>0.01711179217746639</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>-0.02177787812470566</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>102685.3605150107</v>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>0.03166745416018824</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>0.02685360515010737</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>14446.400390625</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>0.05417399231063924</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>-0.02732038716053187</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>101717.1238252686</v>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>-0.009429159958985744</v>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>0.01717123825268585</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>14493.099609375</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>0.05758169945818747</v>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>-0.04041046120550162</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>100070.5429599663</v>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>-0.01618784333826406</v>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>0.0007054295996633542</v>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>14421.2001953125</v>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>0.05233509889904409</v>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>-0.05162966929938073</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>103232.5710170966</v>
+      </c>
+      <c r="C15" s="4" t="n">
+        <v>0.03159799041357481</v>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>0.03232571017096575</v>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>14827.400390625</v>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>0.08197609388682126</v>
+      </c>
+      <c r="G15" s="4" t="n">
+        <v>-0.04965038371585551</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>101665.535802718</v>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>-0.0151796588900126</v>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>0.01665535802718043</v>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>14734.5</v>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>0.07519702276707529</v>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>-0.05854166473989486</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="n">
+        <v>46195</v>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>101579.9132001645</v>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>-0.0008421989013038811</v>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>0.01579913200164529</v>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>14729.7001953125</v>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>0.07484677432227826</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>-0.05904764232063298</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G2"/>
+  <autoFilter ref="A1:G17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -884,7 +1265,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -921,19 +1302,26 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Amaç stratejinin BIST100’e göre performansını takip etmektir.</t>
+          <t>Amaç stratejinin BIST100'e göre performansını takip etmektir.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Bir ay boyunca aynı 3 hisse takip edilir.</t>
+          <t>Portföy reports/tracking_state.json içinden okunur.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Sonraki çalıştırmalarda yeni hisse seçilmez.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:A6"/>
+  <autoFilter ref="A1:A7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>